<commit_message>
Correct ADR measure labels
</commit_message>
<xml_diff>
--- a/2 Output/Phase1_Baseline_Executive/tables/phase1_baseline_all_item_tabulations.xlsx
+++ b/2 Output/Phase1_Baseline_Executive/tables/phase1_baseline_all_item_tabulations.xlsx
@@ -3353,10 +3353,10 @@
     <t>ADR practice score: follow-up after mediation</t>
   </si>
   <si>
-    <t>Appropriate response to non-compliance with mediated agreement</t>
-  </si>
-  <si>
-    <t>Knowledge of when ADR is not appropriate</t>
+    <t>Reported frequency of compliance with mediated agreements</t>
+  </si>
+  <si>
+    <t>Perceived prevention of escalation to police or courts</t>
   </si>
   <si>
     <t>Enumerator verification: In the records seen today, is there any written evidenc</t>

</xml_diff>